<commit_message>
Align KPI forms with country scope
</commit_message>
<xml_diff>
--- a/kobo_forms/PMS_GMC_Formulaire_2_Donnees_Calcul_Journalieres_2026.xlsx
+++ b/kobo_forms/PMS_GMC_Formulaire_2_Donnees_Calcul_Journalieres_2026.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Recfce0ae14474a5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R58e02f6060f54a58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R1ce4c5eb51b84779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rbf806be38b8c45a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R63e4ead7fa714089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R77bd5cac6d164c52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -576,14 +576,14 @@
       <x:c r="C2" s="21" t="str">
         <x:v>Debut</x:v>
       </x:c>
-      <x:c r="D2" s="21" t="str"/>
-      <x:c r="E2" s="21" t="str"/>
-      <x:c r="F2" s="21" t="str"/>
-      <x:c r="G2" s="21" t="str"/>
-      <x:c r="H2" s="21" t="str"/>
-      <x:c r="I2" s="21" t="str"/>
-      <x:c r="J2" s="21" t="str"/>
-      <x:c r="K2" s="22" t="str"/>
+      <x:c r="D2" s="21"/>
+      <x:c r="E2" s="21"/>
+      <x:c r="F2" s="21"/>
+      <x:c r="G2" s="21"/>
+      <x:c r="H2" s="21"/>
+      <x:c r="I2" s="21"/>
+      <x:c r="J2" s="21"/>
+      <x:c r="K2" s="22"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="23" t="str">
@@ -595,14 +595,14 @@
       <x:c r="C3" s="24" t="str">
         <x:v>Fin</x:v>
       </x:c>
-      <x:c r="D3" s="24" t="str"/>
-      <x:c r="E3" s="24" t="str"/>
-      <x:c r="F3" s="24" t="str"/>
-      <x:c r="G3" s="24" t="str"/>
-      <x:c r="H3" s="24" t="str"/>
-      <x:c r="I3" s="24" t="str"/>
-      <x:c r="J3" s="24" t="str"/>
-      <x:c r="K3" s="25" t="str"/>
+      <x:c r="D3" s="24"/>
+      <x:c r="E3" s="24"/>
+      <x:c r="F3" s="24"/>
+      <x:c r="G3" s="24"/>
+      <x:c r="H3" s="24"/>
+      <x:c r="I3" s="24"/>
+      <x:c r="J3" s="24"/>
+      <x:c r="K3" s="25"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="23" t="str">
@@ -614,14 +614,14 @@
       <x:c r="C4" s="24" t="str">
         <x:v>Date de soumission</x:v>
       </x:c>
-      <x:c r="D4" s="24" t="str"/>
-      <x:c r="E4" s="24" t="str"/>
-      <x:c r="F4" s="24" t="str"/>
-      <x:c r="G4" s="24" t="str"/>
-      <x:c r="H4" s="24" t="str"/>
-      <x:c r="I4" s="24" t="str"/>
-      <x:c r="J4" s="24" t="str"/>
-      <x:c r="K4" s="25" t="str"/>
+      <x:c r="D4" s="24"/>
+      <x:c r="E4" s="24"/>
+      <x:c r="F4" s="24"/>
+      <x:c r="G4" s="24"/>
+      <x:c r="H4" s="24"/>
+      <x:c r="I4" s="24"/>
+      <x:c r="J4" s="24"/>
+      <x:c r="K4" s="25"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="23" t="str">
@@ -639,16 +639,16 @@
       <x:c r="E5" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F5" s="24" t="str"/>
-      <x:c r="G5" s="24" t="str"/>
+      <x:c r="F5" s="24"/>
+      <x:c r="G5" s="24"/>
       <x:c r="H5" s="24" t="str">
         <x:v>. &lt;= today()</x:v>
       </x:c>
       <x:c r="I5" s="24" t="str">
         <x:v>La date de collecte ne peut pas etre dans le futur.</x:v>
       </x:c>
-      <x:c r="J5" s="24" t="str"/>
-      <x:c r="K5" s="25" t="str"/>
+      <x:c r="J5" s="24"/>
+      <x:c r="K5" s="25"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="23" t="str">
@@ -657,17 +657,17 @@
       <x:c r="B6" s="24" t="str">
         <x:v>periode_reporting</x:v>
       </x:c>
-      <x:c r="C6" s="24" t="str"/>
-      <x:c r="D6" s="24" t="str"/>
-      <x:c r="E6" s="24" t="str"/>
-      <x:c r="F6" s="24" t="str"/>
+      <x:c r="C6" s="24"/>
+      <x:c r="D6" s="24"/>
+      <x:c r="E6" s="24"/>
+      <x:c r="F6" s="24"/>
       <x:c r="G6" s="24" t="str">
         <x:v>format-date(${date_collecte}, '%Y-%m-%d')</x:v>
       </x:c>
-      <x:c r="H6" s="24" t="str"/>
-      <x:c r="I6" s="24" t="str"/>
-      <x:c r="J6" s="24" t="str"/>
-      <x:c r="K6" s="25" t="str"/>
+      <x:c r="H6" s="24"/>
+      <x:c r="I6" s="24"/>
+      <x:c r="J6" s="24"/>
+      <x:c r="K6" s="25"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="23" t="str">
@@ -679,16 +679,16 @@
       <x:c r="C7" s="24" t="str">
         <x:v>Pays / Filiale</x:v>
       </x:c>
-      <x:c r="D7" s="24" t="str"/>
+      <x:c r="D7" s="24"/>
       <x:c r="E7" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="str"/>
-      <x:c r="G7" s="24" t="str"/>
-      <x:c r="H7" s="24" t="str"/>
-      <x:c r="I7" s="24" t="str"/>
-      <x:c r="J7" s="24" t="str"/>
-      <x:c r="K7" s="25" t="str"/>
+      <x:c r="F7" s="24"/>
+      <x:c r="G7" s="24"/>
+      <x:c r="H7" s="24"/>
+      <x:c r="I7" s="24"/>
+      <x:c r="J7" s="24"/>
+      <x:c r="K7" s="25"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="23" t="str">
@@ -706,12 +706,12 @@
       <x:c r="E8" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F8" s="24" t="str"/>
-      <x:c r="G8" s="24" t="str"/>
-      <x:c r="H8" s="24" t="str"/>
-      <x:c r="I8" s="24" t="str"/>
-      <x:c r="J8" s="24" t="str"/>
-      <x:c r="K8" s="25" t="str"/>
+      <x:c r="F8" s="24"/>
+      <x:c r="G8" s="24"/>
+      <x:c r="H8" s="24"/>
+      <x:c r="I8" s="24"/>
+      <x:c r="J8" s="24"/>
+      <x:c r="K8" s="25"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="23" t="str">
@@ -729,12 +729,12 @@
       <x:c r="E9" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F9" s="24" t="str"/>
-      <x:c r="G9" s="24" t="str"/>
-      <x:c r="H9" s="24" t="str"/>
-      <x:c r="I9" s="24" t="str"/>
-      <x:c r="J9" s="24" t="str"/>
-      <x:c r="K9" s="25" t="str"/>
+      <x:c r="F9" s="24"/>
+      <x:c r="G9" s="24"/>
+      <x:c r="H9" s="24"/>
+      <x:c r="I9" s="24"/>
+      <x:c r="J9" s="24"/>
+      <x:c r="K9" s="25"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="23" t="str">
@@ -752,12 +752,12 @@
       <x:c r="E10" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F10" s="24" t="str"/>
-      <x:c r="G10" s="24" t="str"/>
-      <x:c r="H10" s="24" t="str"/>
-      <x:c r="I10" s="24" t="str"/>
-      <x:c r="J10" s="24" t="str"/>
-      <x:c r="K10" s="25" t="str"/>
+      <x:c r="F10" s="24"/>
+      <x:c r="G10" s="24"/>
+      <x:c r="H10" s="24"/>
+      <x:c r="I10" s="24"/>
+      <x:c r="J10" s="24"/>
+      <x:c r="K10" s="25"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="23" t="str">
@@ -769,16 +769,16 @@
       <x:c r="C11" s="24" t="str">
         <x:v>Valeur collectee</x:v>
       </x:c>
-      <x:c r="D11" s="24" t="str"/>
+      <x:c r="D11" s="24"/>
       <x:c r="E11" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F11" s="24" t="str"/>
-      <x:c r="G11" s="24" t="str"/>
-      <x:c r="H11" s="24" t="str"/>
-      <x:c r="I11" s="24" t="str"/>
-      <x:c r="J11" s="24" t="str"/>
-      <x:c r="K11" s="25" t="str"/>
+      <x:c r="F11" s="24"/>
+      <x:c r="G11" s="24"/>
+      <x:c r="H11" s="24"/>
+      <x:c r="I11" s="24"/>
+      <x:c r="J11" s="24"/>
+      <x:c r="K11" s="25"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="23" t="str">
@@ -790,14 +790,14 @@
       <x:c r="C12" s="24" t="str">
         <x:v>Unite de la valeur</x:v>
       </x:c>
-      <x:c r="D12" s="24" t="str"/>
-      <x:c r="E12" s="24" t="str"/>
-      <x:c r="F12" s="24" t="str"/>
-      <x:c r="G12" s="24" t="str"/>
-      <x:c r="H12" s="24" t="str"/>
-      <x:c r="I12" s="24" t="str"/>
-      <x:c r="J12" s="24" t="str"/>
-      <x:c r="K12" s="25" t="str"/>
+      <x:c r="D12" s="24"/>
+      <x:c r="E12" s="24"/>
+      <x:c r="F12" s="24"/>
+      <x:c r="G12" s="24"/>
+      <x:c r="H12" s="24"/>
+      <x:c r="I12" s="24"/>
+      <x:c r="J12" s="24"/>
+      <x:c r="K12" s="25"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="23" t="str">
@@ -809,16 +809,16 @@
       <x:c r="C13" s="24" t="str">
         <x:v>Frequence de collecte</x:v>
       </x:c>
-      <x:c r="D13" s="24" t="str"/>
-      <x:c r="E13" s="24" t="str"/>
+      <x:c r="D13" s="24"/>
+      <x:c r="E13" s="24"/>
       <x:c r="F13" s="24" t="str">
         <x:v>journalier</x:v>
       </x:c>
-      <x:c r="G13" s="24" t="str"/>
-      <x:c r="H13" s="24" t="str"/>
-      <x:c r="I13" s="24" t="str"/>
-      <x:c r="J13" s="24" t="str"/>
-      <x:c r="K13" s="25" t="str"/>
+      <x:c r="G13" s="24"/>
+      <x:c r="H13" s="24"/>
+      <x:c r="I13" s="24"/>
+      <x:c r="J13" s="24"/>
+      <x:c r="K13" s="25"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="23" t="str">
@@ -830,18 +830,18 @@
       <x:c r="C14" s="24" t="str">
         <x:v>Validation hierarchique</x:v>
       </x:c>
-      <x:c r="D14" s="24" t="str"/>
+      <x:c r="D14" s="24"/>
       <x:c r="E14" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="F14" s="24" t="str">
         <x:v>a_valider</x:v>
       </x:c>
-      <x:c r="G14" s="24" t="str"/>
-      <x:c r="H14" s="24" t="str"/>
-      <x:c r="I14" s="24" t="str"/>
-      <x:c r="J14" s="24" t="str"/>
-      <x:c r="K14" s="25" t="str"/>
+      <x:c r="G14" s="24"/>
+      <x:c r="H14" s="24"/>
+      <x:c r="I14" s="24"/>
+      <x:c r="J14" s="24"/>
+      <x:c r="K14" s="25"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="23" t="str">
@@ -856,13 +856,13 @@
       <x:c r="D15" s="24" t="str">
         <x:v>Systeme, fichier, export ou responsable source.</x:v>
       </x:c>
-      <x:c r="E15" s="24" t="str"/>
-      <x:c r="F15" s="24" t="str"/>
-      <x:c r="G15" s="24" t="str"/>
-      <x:c r="H15" s="24" t="str"/>
-      <x:c r="I15" s="24" t="str"/>
-      <x:c r="J15" s="24" t="str"/>
-      <x:c r="K15" s="25" t="str"/>
+      <x:c r="E15" s="24"/>
+      <x:c r="F15" s="24"/>
+      <x:c r="G15" s="24"/>
+      <x:c r="H15" s="24"/>
+      <x:c r="I15" s="24"/>
+      <x:c r="J15" s="24"/>
+      <x:c r="K15" s="25"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="23" t="str">
@@ -874,14 +874,14 @@
       <x:c r="C16" s="24" t="str">
         <x:v>Responsable de la donnee</x:v>
       </x:c>
-      <x:c r="D16" s="24" t="str"/>
-      <x:c r="E16" s="24" t="str"/>
-      <x:c r="F16" s="24" t="str"/>
-      <x:c r="G16" s="24" t="str"/>
-      <x:c r="H16" s="24" t="str"/>
-      <x:c r="I16" s="24" t="str"/>
-      <x:c r="J16" s="24" t="str"/>
-      <x:c r="K16" s="25" t="str"/>
+      <x:c r="D16" s="24"/>
+      <x:c r="E16" s="24"/>
+      <x:c r="F16" s="24"/>
+      <x:c r="G16" s="24"/>
+      <x:c r="H16" s="24"/>
+      <x:c r="I16" s="24"/>
+      <x:c r="J16" s="24"/>
+      <x:c r="K16" s="25"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="23" t="str">
@@ -893,13 +893,13 @@
       <x:c r="C17" s="24" t="str">
         <x:v>Commentaire</x:v>
       </x:c>
-      <x:c r="D17" s="24" t="str"/>
-      <x:c r="E17" s="24" t="str"/>
-      <x:c r="F17" s="24" t="str"/>
-      <x:c r="G17" s="24" t="str"/>
-      <x:c r="H17" s="24" t="str"/>
-      <x:c r="I17" s="24" t="str"/>
-      <x:c r="J17" s="24" t="str"/>
+      <x:c r="D17" s="24"/>
+      <x:c r="E17" s="24"/>
+      <x:c r="F17" s="24"/>
+      <x:c r="G17" s="24"/>
+      <x:c r="H17" s="24"/>
+      <x:c r="I17" s="24"/>
+      <x:c r="J17" s="24"/>
       <x:c r="K17" s="25" t="str">
         <x:v>multiline</x:v>
       </x:c>
@@ -917,13 +917,13 @@
       <x:c r="D18" s="24" t="str">
         <x:v>Optionnel : fichier source, capture ou justificatif.</x:v>
       </x:c>
-      <x:c r="E18" s="24" t="str"/>
-      <x:c r="F18" s="24" t="str"/>
-      <x:c r="G18" s="24" t="str"/>
-      <x:c r="H18" s="24" t="str"/>
-      <x:c r="I18" s="24" t="str"/>
-      <x:c r="J18" s="24" t="str"/>
-      <x:c r="K18" s="25" t="str"/>
+      <x:c r="E18" s="24"/>
+      <x:c r="F18" s="24"/>
+      <x:c r="G18" s="24"/>
+      <x:c r="H18" s="24"/>
+      <x:c r="I18" s="24"/>
+      <x:c r="J18" s="24"/>
+      <x:c r="K18" s="25"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="26" t="str">
@@ -932,17 +932,17 @@
       <x:c r="B19" s="27" t="str">
         <x:v>cle_pms_calcul</x:v>
       </x:c>
-      <x:c r="C19" s="27" t="str"/>
-      <x:c r="D19" s="27" t="str"/>
-      <x:c r="E19" s="27" t="str"/>
-      <x:c r="F19" s="27" t="str"/>
+      <x:c r="C19" s="27"/>
+      <x:c r="D19" s="27"/>
+      <x:c r="E19" s="27"/>
+      <x:c r="F19" s="27"/>
       <x:c r="G19" s="27" t="str">
-        <x:v>concat(${pole_id}, '|', ${id_kpi}, '|', ${periode_reporting})</x:v>
-      </x:c>
-      <x:c r="H19" s="27" t="str"/>
-      <x:c r="I19" s="27" t="str"/>
-      <x:c r="J19" s="27" t="str"/>
-      <x:c r="K19" s="28" t="str"/>
+        <x:v>concat(${filiale}, '|', ${pole_id}, '|', ${id_kpi}, '|', ${periode_reporting})</x:v>
+      </x:c>
+      <x:c r="H19" s="27"/>
+      <x:c r="I19" s="27"/>
+      <x:c r="J19" s="27"/>
+      <x:c r="K19" s="28"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1655,7 +1655,7 @@
         <x:v>pms_gmc_donnees_calcul_journalieres_2026</x:v>
       </x:c>
       <x:c r="C2" s="30" t="str">
-        <x:v>20260718</x:v>
+        <x:v>20260720</x:v>
       </x:c>
       <x:c r="D2" s="31" t="str">
         <x:v>Francais</x:v>

</xml_diff>